<commit_message>
chage excel sheet values
</commit_message>
<xml_diff>
--- a/Interest_on_Borrowings_2025.xlsx
+++ b/Interest_on_Borrowings_2025.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="11">
   <si>
     <t>Bank Name</t>
   </si>
@@ -39,6 +39,15 @@
   </si>
   <si>
     <t>Jan-2025</t>
+  </si>
+  <si>
+    <t>Feb-2025</t>
+  </si>
+  <si>
+    <t>Mar-2025</t>
+  </si>
+  <si>
+    <t>Apr-2025</t>
   </si>
 </sst>
 </file>
@@ -127,23 +136,41 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Bank-wise Summary'!$A$2</c:f>
+              <c:f>'Bank-wise Summary'!$A$2:$A$5</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>Jan-2025</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb-2025</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar-2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr-2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Bank-wise Summary'!$B$2</c:f>
+              <c:f>'Bank-wise Summary'!$B$2:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>10000</c:v>
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5200</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -160,23 +187,41 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Bank-wise Summary'!$A$2</c:f>
+              <c:f>'Bank-wise Summary'!$A$2:$A$5</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>Jan-2025</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb-2025</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar-2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr-2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Bank-wise Summary'!$C$2</c:f>
+              <c:f>'Bank-wise Summary'!$C$2:$C$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>10000</c:v>
+                  <c:v>2500</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2600</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -299,23 +344,41 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Bank-wise Summary'!$A$2</c:f>
+              <c:f>'Bank-wise Summary'!$A$2:$A$5</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>Jan-2025</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb-2025</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar-2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr-2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Bank-wise Summary'!$B$2</c:f>
+              <c:f>'Bank-wise Summary'!$B$2:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>10000</c:v>
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5200</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -329,23 +392,41 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Bank-wise Summary'!$A$2</c:f>
+              <c:f>'Bank-wise Summary'!$A$2:$A$5</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>Jan-2025</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb-2025</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar-2025</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr-2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Bank-wise Summary'!$C$2</c:f>
+              <c:f>'Bank-wise Summary'!$C$2:$C$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>10000</c:v>
+                  <c:v>2500</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2600</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -488,10 +569,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>10000</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10000</c:v>
+                  <c:v>2500</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -904,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -946,13 +1027,13 @@
         <v>6</v>
       </c>
       <c r="B3" s="1">
-        <v>45673</v>
+        <v>45677</v>
       </c>
       <c r="C3">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="D3">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -963,16 +1044,16 @@
         <v>5</v>
       </c>
       <c r="B4" s="1">
-        <v>45674</v>
+        <v>45703</v>
       </c>
       <c r="C4">
         <v>1000000</v>
       </c>
       <c r="D4">
-        <v>5000</v>
+        <v>5200</v>
       </c>
       <c r="E4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -980,16 +1061,67 @@
         <v>6</v>
       </c>
       <c r="B5" s="1">
-        <v>45675</v>
+        <v>45708</v>
       </c>
       <c r="C5">
+        <v>500000</v>
+      </c>
+      <c r="D5">
+        <v>2600</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>45731</v>
+      </c>
+      <c r="C6">
         <v>1000000</v>
       </c>
-      <c r="D5">
-        <v>5000</v>
-      </c>
-      <c r="E5" t="s">
-        <v>7</v>
+      <c r="D6">
+        <v>5100</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1">
+        <v>45736</v>
+      </c>
+      <c r="C7">
+        <v>500000</v>
+      </c>
+      <c r="D7">
+        <v>2700</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1">
+        <v>45762</v>
+      </c>
+      <c r="C8">
+        <v>1000000</v>
+      </c>
+      <c r="D8">
+        <v>5300</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -999,7 +1131,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1018,10 +1150,43 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="C2">
-        <v>10000</v>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>5200</v>
+      </c>
+      <c r="C3">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>5100</v>
+      </c>
+      <c r="C4">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>5300</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>